<commit_message>
Actualiza chequeo de adjuntos rotos
</commit_message>
<xml_diff>
--- a/reportes/entradas_a_revisar.xlsx
+++ b/reportes/entradas_a_revisar.xlsx
@@ -556,15 +556,13 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr"/>
+      <c r="E2" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -584,15 +582,13 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="8" t="n">
+        <v>225706</v>
+      </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -612,15 +608,13 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="8" t="n">
+        <v>525856</v>
+      </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -640,15 +634,13 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="8" t="n">
+        <v>266113</v>
+      </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -668,15 +660,13 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="8" t="n">
+        <v>22027092</v>
+      </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -696,15 +686,13 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="8" t="n">
+        <v>29548</v>
+      </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -724,15 +712,13 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="8" t="n">
+        <v>93194</v>
+      </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -752,15 +738,13 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -780,15 +764,13 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="8" t="n">
+        <v>66244</v>
+      </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -808,15 +790,13 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -836,15 +816,13 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="8" t="n">
+        <v>308626</v>
+      </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -864,15 +842,13 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="8" t="n">
+        <v>100519</v>
+      </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -892,15 +868,13 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="8" t="n">
+        <v>269204</v>
+      </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -920,15 +894,13 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="8" t="n">
+        <v>101840</v>
+      </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -948,15 +920,13 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="8" t="n">
+        <v>66641</v>
+      </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -976,15 +946,13 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="8" t="n">
+        <v>75481</v>
+      </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1004,15 +972,13 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr"/>
+      <c r="E18" s="8" t="n">
+        <v>144527</v>
+      </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1032,15 +998,13 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
+      <c r="E19" s="8" t="n">
+        <v>71677</v>
+      </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1060,15 +1024,13 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr"/>
+      <c r="E20" s="8" t="n">
+        <v>77244</v>
+      </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1088,15 +1050,13 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr"/>
+      <c r="E21" s="8" t="n">
+        <v>6781749</v>
+      </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1116,15 +1076,13 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr"/>
+      <c r="E22" s="8" t="n">
+        <v>929482</v>
+      </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1144,15 +1102,13 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr"/>
+      <c r="E23" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1172,15 +1128,13 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr"/>
+      <c r="E24" s="8" t="n">
+        <v>96389</v>
+      </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1200,15 +1154,13 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr"/>
+      <c r="E25" s="8" t="n">
+        <v>255212</v>
+      </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1228,15 +1180,13 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr"/>
+      <c r="E26" s="8" t="n">
+        <v>340220</v>
+      </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1256,15 +1206,13 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr"/>
+      <c r="E27" s="8" t="n">
+        <v>6598</v>
+      </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1284,15 +1232,13 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr"/>
+      <c r="E28" s="8" t="n">
+        <v>800486</v>
+      </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1312,15 +1258,13 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr"/>
+      <c r="E29" s="8" t="n">
+        <v>67940</v>
+      </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1340,15 +1284,13 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr"/>
+      <c r="E30" s="8" t="n">
+        <v>2389738</v>
+      </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1368,15 +1310,13 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr"/>
+      <c r="E31" s="8" t="n">
+        <v>333899</v>
+      </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1396,15 +1336,13 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr"/>
+      <c r="E32" s="8" t="n">
+        <v>340841</v>
+      </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1424,15 +1362,13 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
+      <c r="E33" s="8" t="n">
+        <v>171169</v>
+      </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1452,15 +1388,13 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="8" t="n">
+        <v>244252</v>
+      </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1480,15 +1414,13 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
+      <c r="E35" s="8" t="n">
+        <v>428565</v>
+      </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1508,15 +1440,13 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr"/>
+      <c r="E36" s="8" t="n">
+        <v>123974</v>
+      </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1536,15 +1466,13 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr"/>
+      <c r="E37" s="8" t="n">
+        <v>778731</v>
+      </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1564,15 +1492,13 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr"/>
+      <c r="E38" s="8" t="n">
+        <v>283214</v>
+      </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1592,15 +1518,13 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr"/>
+      <c r="E39" s="8" t="n">
+        <v>732192</v>
+      </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1620,15 +1544,13 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr"/>
+      <c r="E40" s="8" t="n">
+        <v>278733</v>
+      </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1648,15 +1570,13 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr"/>
+      <c r="E41" s="8" t="n">
+        <v>109006</v>
+      </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1676,15 +1596,13 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr"/>
+      <c r="E42" s="8" t="n">
+        <v>224118</v>
+      </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1704,15 +1622,13 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr"/>
+      <c r="E43" s="8" t="n">
+        <v>242092</v>
+      </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1732,15 +1648,13 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr"/>
+      <c r="E44" s="8" t="n">
+        <v>381932</v>
+      </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1760,15 +1674,13 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr"/>
+      <c r="E45" s="8" t="n">
+        <v>113459</v>
+      </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1788,15 +1700,13 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr"/>
+      <c r="E46" s="8" t="n">
+        <v>1397760</v>
+      </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1816,15 +1726,13 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
+      <c r="E47" s="8" t="n">
+        <v>82457</v>
+      </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1844,15 +1752,13 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr"/>
+      <c r="E48" s="8" t="n">
+        <v>32256</v>
+      </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1872,15 +1778,13 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr"/>
+      <c r="E49" s="8" t="n">
+        <v>340100</v>
+      </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1900,15 +1804,13 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr"/>
+      <c r="E50" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1928,15 +1830,13 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr"/>
+      <c r="E51" s="8" t="n">
+        <v>1559387</v>
+      </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1956,15 +1856,13 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr"/>
+      <c r="E52" s="8" t="n">
+        <v>139317</v>
+      </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -1984,15 +1882,13 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr"/>
+      <c r="E53" s="8" t="n">
+        <v>1389397</v>
+      </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2012,15 +1908,13 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr"/>
+      <c r="E54" s="8" t="n">
+        <v>464657</v>
+      </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2040,15 +1934,13 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr"/>
+      <c r="E55" s="8" t="n">
+        <v>109006</v>
+      </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2068,15 +1960,13 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr"/>
+      <c r="E56" s="8" t="n">
+        <v>136293</v>
+      </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2096,15 +1986,13 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr"/>
+      <c r="E57" s="8" t="n">
+        <v>101040</v>
+      </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2124,15 +2012,13 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr"/>
+      <c r="E58" s="8" t="n">
+        <v>99253</v>
+      </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2152,15 +2038,13 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr"/>
+      <c r="E59" s="8" t="n">
+        <v>262604</v>
+      </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2180,15 +2064,13 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D60" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr"/>
+      <c r="E60" s="8" t="n">
+        <v>615458</v>
+      </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2208,15 +2090,13 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr"/>
+      <c r="E61" s="8" t="n">
+        <v>407459</v>
+      </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2236,15 +2116,13 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr"/>
+      <c r="E62" s="8" t="n">
+        <v>78730</v>
+      </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2264,15 +2142,13 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr"/>
+      <c r="E63" s="8" t="n">
+        <v>102597</v>
+      </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2292,15 +2168,13 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr"/>
+      <c r="E64" s="8" t="n">
+        <v>130063</v>
+      </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2320,15 +2194,13 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D65" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr"/>
+      <c r="E65" s="8" t="n">
+        <v>334057</v>
+      </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2348,15 +2220,13 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D66" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr"/>
+      <c r="E66" s="8" t="n">
+        <v>680920</v>
+      </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2376,15 +2246,13 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr"/>
+      <c r="E67" s="8" t="n">
+        <v>268458</v>
+      </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2404,15 +2272,13 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E68" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr"/>
+      <c r="E68" s="8" t="n">
+        <v>371830</v>
+      </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2432,15 +2298,13 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D69" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr"/>
+      <c r="E69" s="8" t="n">
+        <v>372060</v>
+      </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2460,15 +2324,13 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D70" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr"/>
+      <c r="E70" s="8" t="n">
+        <v>606742</v>
+      </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2488,15 +2350,13 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr"/>
+      <c r="E71" s="8" t="n">
+        <v>263854</v>
+      </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2516,15 +2376,13 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D72" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr"/>
+      <c r="E72" s="8" t="n">
+        <v>173396</v>
+      </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2544,15 +2402,13 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr"/>
+      <c r="E73" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2572,15 +2428,13 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D74" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr"/>
+      <c r="E74" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2600,15 +2454,13 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr"/>
+      <c r="E75" s="8" t="n">
+        <v>1000901</v>
+      </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2628,15 +2480,13 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D76" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr"/>
+      <c r="E76" s="8" t="n">
+        <v>2450284</v>
+      </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2656,15 +2506,13 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr"/>
+      <c r="E77" s="8" t="n">
+        <v>27358</v>
+      </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2684,15 +2532,13 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E78" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr"/>
+      <c r="E78" s="8" t="n">
+        <v>101840</v>
+      </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2712,15 +2558,13 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr"/>
+      <c r="E79" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2740,15 +2584,13 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E80" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr"/>
+      <c r="E80" s="8" t="n">
+        <v>201941</v>
+      </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2768,15 +2610,13 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr"/>
+      <c r="E81" s="8" t="n">
+        <v>118412</v>
+      </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2796,15 +2636,13 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E82" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr"/>
+      <c r="E82" s="8" t="n">
+        <v>436276</v>
+      </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2824,15 +2662,13 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D83" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E83" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr"/>
+      <c r="E83" s="8" t="n">
+        <v>159181</v>
+      </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2852,15 +2688,13 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D84" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E84" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr"/>
+      <c r="E84" s="8" t="n">
+        <v>963884</v>
+      </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2880,15 +2714,13 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr"/>
+      <c r="E85" s="8" t="n">
+        <v>181923</v>
+      </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2908,15 +2740,13 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E86" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr"/>
+      <c r="E86" s="8" t="n">
+        <v>196912</v>
+      </c>
       <c r="F86" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2936,15 +2766,13 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E87" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr"/>
+      <c r="E87" s="8" t="n">
+        <v>116798</v>
+      </c>
       <c r="F87" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2964,15 +2792,13 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E88" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr"/>
+      <c r="E88" s="8" t="n">
+        <v>184464</v>
+      </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -2992,15 +2818,13 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E89" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr"/>
+      <c r="E89" s="8" t="n">
+        <v>4767626</v>
+      </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3020,15 +2844,13 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E90" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr"/>
+      <c r="E90" s="8" t="n">
+        <v>105472</v>
+      </c>
       <c r="F90" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3048,15 +2870,13 @@
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E91" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr"/>
+      <c r="E91" s="8" t="n">
+        <v>253823</v>
+      </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3076,15 +2896,13 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E92" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr"/>
+      <c r="E92" s="8" t="n">
+        <v>150820</v>
+      </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3104,15 +2922,13 @@
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D93" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E93" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr"/>
+      <c r="E93" s="8" t="n">
+        <v>1987313</v>
+      </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3132,15 +2948,13 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D94" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E94" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr"/>
+      <c r="E94" s="8" t="n">
+        <v>528084</v>
+      </c>
       <c r="F94" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3160,15 +2974,13 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E95" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr"/>
+      <c r="E95" s="8" t="n">
+        <v>36718</v>
+      </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3188,15 +3000,13 @@
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D96" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E96" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr"/>
+      <c r="E96" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3216,15 +3026,13 @@
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E97" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr"/>
+      <c r="E97" s="8" t="n">
+        <v>68096</v>
+      </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3244,15 +3052,13 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E98" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr"/>
+      <c r="E98" s="8" t="n">
+        <v>42496</v>
+      </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3272,15 +3078,13 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D99" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E99" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr"/>
+      <c r="E99" s="8" t="n">
+        <v>577524</v>
+      </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3300,15 +3104,13 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D100" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E100" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr"/>
+      <c r="E100" s="8" t="n">
+        <v>46</v>
+      </c>
       <c r="F100" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3328,15 +3130,13 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D101" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E101" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr"/>
+      <c r="E101" s="8" t="n">
+        <v>242092</v>
+      </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3356,15 +3156,13 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D102" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E102" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="inlineStr"/>
+      <c r="E102" s="8" t="n">
+        <v>101840</v>
+      </c>
       <c r="F102" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3384,15 +3182,13 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D103" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E103" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr"/>
+      <c r="E103" s="8" t="n">
+        <v>101840</v>
+      </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3412,15 +3208,13 @@
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D104" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E104" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr"/>
+      <c r="E104" s="8" t="n">
+        <v>67353</v>
+      </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3440,15 +3234,13 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr"/>
+      <c r="E105" s="8" t="n">
+        <v>60416</v>
+      </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3468,15 +3260,13 @@
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D106" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E106" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="inlineStr"/>
+      <c r="E106" s="8" t="n">
+        <v>35308</v>
+      </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3496,15 +3286,13 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E107" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr"/>
+      <c r="E107" s="8" t="n">
+        <v>14744</v>
+      </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3524,15 +3312,13 @@
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D108" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E108" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="inlineStr"/>
+      <c r="E108" s="8" t="n">
+        <v>210683</v>
+      </c>
       <c r="F108" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3552,15 +3338,13 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D109" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E109" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr"/>
+      <c r="E109" s="8" t="n">
+        <v>46592</v>
+      </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3580,15 +3364,13 @@
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E110" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="inlineStr"/>
+      <c r="E110" s="8" t="n">
+        <v>17975</v>
+      </c>
       <c r="F110" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3608,15 +3390,13 @@
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D111" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E111" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D111" s="7" t="inlineStr"/>
+      <c r="E111" s="8" t="n">
+        <v>165064</v>
+      </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3636,15 +3416,13 @@
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D112" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E112" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="inlineStr"/>
+      <c r="E112" s="8" t="n">
+        <v>74575</v>
+      </c>
       <c r="F112" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3664,15 +3442,13 @@
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D113" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E113" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr"/>
+      <c r="E113" s="8" t="n">
+        <v>198064</v>
+      </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3692,15 +3468,13 @@
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D114" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E114" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr"/>
+      <c r="E114" s="8" t="n">
+        <v>78401</v>
+      </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3720,15 +3494,13 @@
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D115" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E115" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr"/>
+      <c r="E115" s="8" t="n">
+        <v>85189</v>
+      </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3748,15 +3520,13 @@
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D116" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E116" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr"/>
+      <c r="E116" s="8" t="n">
+        <v>213372</v>
+      </c>
       <c r="F116" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3776,15 +3546,13 @@
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D117" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E117" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr"/>
+      <c r="E117" s="8" t="n">
+        <v>29209</v>
+      </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3804,15 +3572,13 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D118" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E118" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr"/>
+      <c r="E118" s="8" t="n">
+        <v>101840</v>
+      </c>
       <c r="F118" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3832,15 +3598,13 @@
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D119" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr"/>
+      <c r="E119" s="8" t="n">
+        <v>156466</v>
+      </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3860,15 +3624,13 @@
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D120" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E120" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr"/>
+      <c r="E120" s="8" t="n">
+        <v>50134</v>
+      </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3888,15 +3650,13 @@
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D121" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E121" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr"/>
+      <c r="E121" s="8" t="n">
+        <v>55356</v>
+      </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3916,15 +3676,13 @@
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D122" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E122" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr"/>
+      <c r="E122" s="8" t="n">
+        <v>68144</v>
+      </c>
       <c r="F122" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3944,15 +3702,13 @@
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D123" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr"/>
+      <c r="E123" s="8" t="n">
+        <v>79872</v>
+      </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -3972,15 +3728,13 @@
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D124" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E124" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="inlineStr"/>
+      <c r="E124" s="8" t="n">
+        <v>580001</v>
+      </c>
       <c r="F124" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4000,15 +3754,13 @@
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D125" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E125" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="inlineStr"/>
+      <c r="E125" s="8" t="n">
+        <v>773471</v>
+      </c>
       <c r="F125" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4028,15 +3780,13 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D126" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E126" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr"/>
+      <c r="E126" s="8" t="n">
+        <v>14848</v>
+      </c>
       <c r="F126" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4056,15 +3806,13 @@
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D127" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E127" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr"/>
+      <c r="E127" s="8" t="n">
+        <v>379658</v>
+      </c>
       <c r="F127" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4084,15 +3832,13 @@
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D128" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E128" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr"/>
+      <c r="E128" s="8" t="n">
+        <v>20891207</v>
+      </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4112,15 +3858,13 @@
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D129" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E129" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr"/>
+      <c r="E129" s="8" t="n">
+        <v>159693</v>
+      </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4140,15 +3884,13 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D130" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E130" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr"/>
+      <c r="E130" s="8" t="n">
+        <v>345489</v>
+      </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4168,15 +3910,13 @@
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D131" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E131" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr"/>
+      <c r="E131" s="8" t="n">
+        <v>286761</v>
+      </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4196,15 +3936,13 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D132" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E132" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="inlineStr"/>
+      <c r="E132" s="8" t="n">
+        <v>299569</v>
+      </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4224,15 +3962,13 @@
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D133" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E133" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="inlineStr"/>
+      <c r="E133" s="8" t="n">
+        <v>56514</v>
+      </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4252,15 +3988,13 @@
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D134" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E134" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="inlineStr"/>
+      <c r="E134" s="8" t="n">
+        <v>41984</v>
+      </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4280,15 +4014,13 @@
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D135" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E135" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr"/>
+      <c r="E135" s="8" t="n">
+        <v>67072</v>
+      </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4308,15 +4040,13 @@
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D136" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E136" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="inlineStr"/>
+      <c r="E136" s="8" t="n">
+        <v>32256</v>
+      </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4336,15 +4066,13 @@
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D137" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E137" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D137" s="7" t="inlineStr"/>
+      <c r="E137" s="8" t="n">
+        <v>44032</v>
+      </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4364,15 +4092,13 @@
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D138" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E138" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr"/>
+      <c r="E138" s="8" t="n">
+        <v>12540</v>
+      </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4392,15 +4118,13 @@
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D139" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E139" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr"/>
+      <c r="E139" s="8" t="n">
+        <v>221083</v>
+      </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4420,15 +4144,13 @@
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D140" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E140" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="inlineStr"/>
+      <c r="E140" s="8" t="n">
+        <v>40448</v>
+      </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4448,15 +4170,13 @@
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D141" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E141" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr"/>
+      <c r="E141" s="8" t="n">
+        <v>73864</v>
+      </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4476,15 +4196,13 @@
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D142" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E142" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="inlineStr"/>
+      <c r="E142" s="8" t="n">
+        <v>233302</v>
+      </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4504,15 +4222,13 @@
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D143" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E143" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr"/>
+      <c r="E143" s="8" t="n">
+        <v>49164</v>
+      </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4532,15 +4248,13 @@
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D144" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E144" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="inlineStr"/>
+      <c r="E144" s="8" t="n">
+        <v>190595</v>
+      </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4560,15 +4274,13 @@
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D145" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E145" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr"/>
+      <c r="E145" s="8" t="n">
+        <v>34685</v>
+      </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4588,15 +4300,13 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D146" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E146" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D146" s="7" t="inlineStr"/>
+      <c r="E146" s="8" t="n">
+        <v>13994</v>
+      </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4616,15 +4326,13 @@
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D147" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E147" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D147" s="7" t="inlineStr"/>
+      <c r="E147" s="8" t="n">
+        <v>847416</v>
+      </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4644,15 +4352,13 @@
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D148" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E148" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="inlineStr"/>
+      <c r="E148" s="8" t="n">
+        <v>191783</v>
+      </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4672,15 +4378,13 @@
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D149" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E149" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D149" s="7" t="inlineStr"/>
+      <c r="E149" s="8" t="n">
+        <v>20133</v>
+      </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4700,15 +4404,13 @@
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D150" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E150" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="inlineStr"/>
+      <c r="E150" s="8" t="n">
+        <v>19143</v>
+      </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>
@@ -4728,15 +4430,13 @@
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D151" s="7" t="inlineStr">
-        <is>
-          <t>No se pudo interpretar el link/handle pegado</t>
-        </is>
-      </c>
-      <c r="E151" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D151" s="7" t="inlineStr"/>
+      <c r="E151" s="8" t="n">
+        <v>146307</v>
+      </c>
       <c r="F151" s="7" t="inlineStr">
         <is>
           <t>2026-07-20</t>

</xml_diff>